<commit_message>
Added revised meta data sheet
</commit_message>
<xml_diff>
--- a/tab_data/master.xlsx
+++ b/tab_data/master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Neurology\Gate_Lab\Boles\als_motor_circuit_visium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0FEB8A-FB56-40AC-A6EC-AB7E4061E07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B158C1F-A498-404D-B004-EF04C85A75CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="345" windowWidth="28125" windowHeight="14700" xr2:uid="{A0B421F2-6A50-41F1-B76E-1758D3072867}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{A0B421F2-6A50-41F1-B76E-1758D3072867}"/>
   </bookViews>
   <sheets>
     <sheet name="sample_prep" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="271">
   <si>
     <t>sample</t>
   </si>
@@ -805,6 +805,51 @@
   </si>
   <si>
     <t>G8</t>
+  </si>
+  <si>
+    <t>JSB171-1</t>
+  </si>
+  <si>
+    <t>JSB171-2</t>
+  </si>
+  <si>
+    <t>JSB171-3</t>
+  </si>
+  <si>
+    <t>JSB171-4</t>
+  </si>
+  <si>
+    <t>JSB171-5</t>
+  </si>
+  <si>
+    <t>JSB171-6</t>
+  </si>
+  <si>
+    <t>JSB171-7</t>
+  </si>
+  <si>
+    <t>JSB171-8</t>
+  </si>
+  <si>
+    <t>JSB171-9</t>
+  </si>
+  <si>
+    <t>E9</t>
+  </si>
+  <si>
+    <t>V56F23-309</t>
+  </si>
+  <si>
+    <t>V56F23-348</t>
+  </si>
+  <si>
+    <t>V56F23-322</t>
+  </si>
+  <si>
+    <t>V56F23-329</t>
+  </si>
+  <si>
+    <t>V56F23-339</t>
   </si>
 </sst>
 </file>
@@ -1309,7 +1354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AB8678F-5950-4B3C-9CF7-0F2CA191A3B8}">
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -2503,7 +2548,7 @@
         <v>15</v>
       </c>
       <c r="J35">
-        <f t="shared" ref="J35:J57" si="2">I35+2</f>
+        <f t="shared" ref="J35:J66" si="2">I35+2</f>
         <v>17</v>
       </c>
       <c r="K35" t="s">
@@ -3291,6 +3336,276 @@
       </c>
       <c r="L57">
         <v>11042</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>256</v>
+      </c>
+      <c r="B58" t="s">
+        <v>101</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G58" t="s">
+        <v>266</v>
+      </c>
+      <c r="H58" t="s">
+        <v>14</v>
+      </c>
+      <c r="I58">
+        <v>12</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="K58" t="s">
+        <v>160</v>
+      </c>
+      <c r="L58">
+        <v>10561</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>257</v>
+      </c>
+      <c r="B59" t="s">
+        <v>152</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G59" t="s">
+        <v>268</v>
+      </c>
+      <c r="H59" t="s">
+        <v>13</v>
+      </c>
+      <c r="I59">
+        <v>13</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="K59" t="s">
+        <v>161</v>
+      </c>
+      <c r="L59">
+        <v>6383</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>258</v>
+      </c>
+      <c r="B60" t="s">
+        <v>203</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G60" t="s">
+        <v>267</v>
+      </c>
+      <c r="H60" t="s">
+        <v>13</v>
+      </c>
+      <c r="I60">
+        <v>14</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="K60" t="s">
+        <v>162</v>
+      </c>
+      <c r="L60">
+        <v>8767</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>259</v>
+      </c>
+      <c r="B61" t="s">
+        <v>134</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G61" t="s">
+        <v>266</v>
+      </c>
+      <c r="H61" t="s">
+        <v>13</v>
+      </c>
+      <c r="I61">
+        <v>12</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="K61" t="s">
+        <v>163</v>
+      </c>
+      <c r="L61">
+        <v>11344</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>260</v>
+      </c>
+      <c r="B62" t="s">
+        <v>169</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G62" t="s">
+        <v>268</v>
+      </c>
+      <c r="H62" t="s">
+        <v>14</v>
+      </c>
+      <c r="I62">
+        <v>13</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="K62" t="s">
+        <v>164</v>
+      </c>
+      <c r="L62">
+        <v>12866</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>261</v>
+      </c>
+      <c r="B63" t="s">
+        <v>127</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G63" t="s">
+        <v>269</v>
+      </c>
+      <c r="H63" t="s">
+        <v>14</v>
+      </c>
+      <c r="I63">
+        <v>12</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="K63" t="s">
+        <v>165</v>
+      </c>
+      <c r="L63">
+        <v>8101</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>262</v>
+      </c>
+      <c r="B64" t="s">
+        <v>168</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G64" t="s">
+        <v>269</v>
+      </c>
+      <c r="H64" t="s">
+        <v>13</v>
+      </c>
+      <c r="I64">
+        <v>13</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="K64" t="s">
+        <v>166</v>
+      </c>
+      <c r="L64">
+        <v>8232</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>263</v>
+      </c>
+      <c r="B65" t="s">
+        <v>98</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G65" t="s">
+        <v>270</v>
+      </c>
+      <c r="H65" t="s">
+        <v>14</v>
+      </c>
+      <c r="I65">
+        <v>11</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="K65" t="s">
+        <v>167</v>
+      </c>
+      <c r="L65">
+        <v>9900</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>264</v>
+      </c>
+      <c r="B66" t="s">
+        <v>129</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G66" t="s">
+        <v>270</v>
+      </c>
+      <c r="H66" t="s">
+        <v>13</v>
+      </c>
+      <c r="I66">
+        <v>12</v>
+      </c>
+      <c r="J66">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="K66" t="s">
+        <v>265</v>
+      </c>
+      <c r="L66">
+        <v>7030</v>
       </c>
     </row>
   </sheetData>

</xml_diff>